<commit_message>
Subo proyecto con la arquitectura con clases
</commit_message>
<xml_diff>
--- a/CronogramaHito1_Grupo6.xlsx
+++ b/CronogramaHito1_Grupo6.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Universidad\Proyecto_Computacion_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Universidad\Proyecto_Computacion_2\proyecto_computacion_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CB9A764-F926-46D5-8493-B5F83806C7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1149978E-B4E8-47F5-B850-4072A0C4626B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7F42FA1D-32E5-43B4-9CD2-D0CD4F373669}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="117">
   <si>
     <t>Tareas base de datos:</t>
   </si>
@@ -524,12 +524,45 @@
   <si>
     <t>Alberto García                                               3h</t>
   </si>
+  <si>
+    <t>Victor Vega                                                       1h</t>
+  </si>
+  <si>
+    <t>Victor Vega / Alberto García                   0.5h/por persona</t>
+  </si>
+  <si>
+    <t>Samuel Sánchez / Victor Vega               1.5h/por persona</t>
+  </si>
+  <si>
+    <t>Samuel Sánchez                                           0.5h</t>
+  </si>
+  <si>
+    <t>Samuel Sánchez / Ivan García               1h/por persona</t>
+  </si>
+  <si>
+    <t>Ivan García                                                        1h</t>
+  </si>
+  <si>
+    <t>Ivan García / Jiale Chen                             1h/por persona</t>
+  </si>
+  <si>
+    <t>Jiale Chen                                                         1h</t>
+  </si>
+  <si>
+    <t>Jiale Chen / Alberto García                     1h/por persona</t>
+  </si>
+  <si>
+    <t>Alberto García                                               1.5h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alberto García                                               </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -701,6 +734,15 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="16"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -761,7 +803,7 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -840,6 +882,8 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="1" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Énfasis5" xfId="2" builtinId="45"/>
@@ -2028,11 +2072,9 @@
         <v>98</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>11</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="F14" s="2"/>
       <c r="G14" s="27"/>
       <c r="H14" s="27"/>
       <c r="I14" s="27"/>
@@ -2046,11 +2088,9 @@
         <v>97</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>13</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="F15" s="2"/>
       <c r="G15" s="27"/>
       <c r="H15" s="27"/>
       <c r="I15" s="27"/>
@@ -2064,11 +2104,9 @@
         <v>96</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>15</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="F16" s="2"/>
       <c r="G16" s="27"/>
       <c r="H16" s="27"/>
       <c r="I16" s="27"/>
@@ -2082,11 +2120,9 @@
         <v>99</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17" s="18" t="s">
-        <v>17</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="F17" s="2"/>
       <c r="G17" s="27"/>
       <c r="H17" s="27"/>
       <c r="I17" s="27"/>
@@ -2100,11 +2136,9 @@
         <v>100</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>19</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="F18" s="2"/>
       <c r="G18" s="27"/>
       <c r="H18" s="27"/>
       <c r="I18" s="27"/>
@@ -2118,11 +2152,9 @@
         <v>101</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>21</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="F19" s="2"/>
       <c r="G19" s="27"/>
       <c r="H19" s="27"/>
       <c r="I19" s="27"/>
@@ -2136,11 +2168,9 @@
         <v>102</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>23</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="F20" s="2"/>
       <c r="G20" s="27"/>
       <c r="H20" s="27"/>
       <c r="I20" s="27"/>
@@ -2154,11 +2184,9 @@
         <v>103</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>25</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="F21" s="2"/>
       <c r="G21" s="27"/>
       <c r="H21" s="27"/>
       <c r="I21" s="27"/>
@@ -2172,11 +2200,9 @@
         <v>104</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="F22" s="18" t="s">
-        <v>27</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="F22" s="2"/>
       <c r="G22" s="27"/>
       <c r="H22" s="27"/>
       <c r="I22" s="27"/>
@@ -2190,12 +2216,10 @@
         <v>105</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="G23" s="27"/>
+        <v>115</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="34"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
     </row>
@@ -2218,10 +2242,10 @@
       <c r="C25" s="27"/>
       <c r="D25" s="27"/>
       <c r="E25" s="18" t="s">
-        <v>11</v>
+        <v>107</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>11</v>
+        <v>107</v>
       </c>
       <c r="G25" s="27"/>
       <c r="H25" s="27"/>
@@ -2234,10 +2258,10 @@
       <c r="C26" s="27"/>
       <c r="D26" s="27"/>
       <c r="E26" s="18" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="G26" s="27"/>
       <c r="H26" s="27"/>
@@ -2250,10 +2274,10 @@
       <c r="C27" s="27"/>
       <c r="D27" s="27"/>
       <c r="E27" s="18" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="G27" s="27"/>
       <c r="H27" s="27"/>
@@ -2266,10 +2290,10 @@
       <c r="C28" s="27"/>
       <c r="D28" s="27"/>
       <c r="E28" s="18" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="G28" s="27"/>
       <c r="H28" s="27"/>
@@ -2282,10 +2306,10 @@
       <c r="C29" s="27"/>
       <c r="D29" s="27"/>
       <c r="E29" s="18" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="F29" s="18" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="G29" s="27"/>
       <c r="H29" s="27"/>
@@ -2298,10 +2322,10 @@
       <c r="C30" s="27"/>
       <c r="D30" s="27"/>
       <c r="E30" s="18" t="s">
-        <v>21</v>
+        <v>111</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>21</v>
+        <v>111</v>
       </c>
       <c r="G30" s="27"/>
       <c r="H30" s="27"/>
@@ -2314,10 +2338,10 @@
       <c r="C31" s="27"/>
       <c r="D31" s="27"/>
       <c r="E31" s="18" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="G31" s="27"/>
       <c r="H31" s="27"/>
@@ -2330,10 +2354,10 @@
       <c r="C32" s="27"/>
       <c r="D32" s="27"/>
       <c r="E32" s="18" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="G32" s="27"/>
       <c r="H32" s="27"/>
@@ -2346,10 +2370,10 @@
       <c r="C33" s="27"/>
       <c r="D33" s="27"/>
       <c r="E33" s="18" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="F33" s="18" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="G33" s="27"/>
       <c r="H33" s="27"/>
@@ -2362,10 +2386,10 @@
       <c r="C34" s="27"/>
       <c r="D34" s="27"/>
       <c r="E34" s="18" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="G34" s="27"/>
       <c r="H34" s="27"/>
@@ -2420,10 +2444,10 @@
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="18" t="s">
-        <v>11</v>
+        <v>107</v>
       </c>
       <c r="G37" s="18" t="s">
-        <v>11</v>
+        <v>107</v>
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
@@ -2436,10 +2460,10 @@
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="18" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="G38" s="18" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -2452,10 +2476,10 @@
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="18" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="G39" s="18" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
@@ -2468,10 +2492,10 @@
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
       <c r="F40" s="18" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="G40" s="18" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -2484,10 +2508,10 @@
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
       <c r="F41" s="18" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="G41" s="18" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
@@ -2500,10 +2524,10 @@
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="18" t="s">
-        <v>21</v>
+        <v>111</v>
       </c>
       <c r="G42" s="18" t="s">
-        <v>21</v>
+        <v>111</v>
       </c>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
@@ -2516,10 +2540,10 @@
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
       <c r="F43" s="18" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="G43" s="18" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
@@ -2532,10 +2556,10 @@
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="18" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="G44" s="18" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
@@ -2548,10 +2572,10 @@
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
       <c r="F45" s="18" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="G45" s="18" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
@@ -2564,10 +2588,10 @@
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
       <c r="F46" s="18" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="G46" s="18" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
@@ -2593,7 +2617,7 @@
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
       <c r="G48" s="18" t="s">
-        <v>11</v>
+        <v>107</v>
       </c>
       <c r="H48" s="18" t="s">
         <v>11</v>
@@ -2609,7 +2633,7 @@
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
       <c r="G49" s="18" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="H49" s="18" t="s">
         <v>13</v>
@@ -2625,7 +2649,7 @@
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
       <c r="G50" s="18" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="H50" s="18" t="s">
         <v>15</v>
@@ -2641,7 +2665,7 @@
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
       <c r="G51" s="18" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="H51" s="18" t="s">
         <v>17</v>
@@ -2658,7 +2682,7 @@
       <c r="E52" s="31"/>
       <c r="F52" s="2"/>
       <c r="G52" s="18" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="H52" s="18" t="s">
         <v>19</v>
@@ -2673,9 +2697,9 @@
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
+      <c r="F53" s="35"/>
       <c r="G53" s="18" t="s">
-        <v>21</v>
+        <v>111</v>
       </c>
       <c r="H53" s="18" t="s">
         <v>21</v>
@@ -2691,7 +2715,7 @@
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
       <c r="G54" s="18" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="H54" s="18" t="s">
         <v>23</v>
@@ -2707,7 +2731,7 @@
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
       <c r="G55" s="18" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="H55" s="18" t="s">
         <v>25</v>
@@ -2723,7 +2747,7 @@
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
       <c r="G56" s="18" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="H56" s="18" t="s">
         <v>27</v>
@@ -2738,8 +2762,12 @@
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
+      <c r="G57" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="H57" s="18" t="s">
+        <v>116</v>
+      </c>
       <c r="I57" s="2"/>
     </row>
     <row r="58" spans="1:9" s="21" customFormat="1" ht="198.75" customHeight="1">

</xml_diff>

<commit_message>
Subo proyecto con la conexion a Ubuntu
</commit_message>
<xml_diff>
--- a/CronogramaHito1_Grupo6.xlsx
+++ b/CronogramaHito1_Grupo6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Universidad\Proyecto_Computacion_2\proyecto_computacion_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1149978E-B4E8-47F5-B850-4072A0C4626B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7811A163-75E0-4373-9141-DE1C985F1AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7F42FA1D-32E5-43B4-9CD2-D0CD4F373669}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="116">
   <si>
     <t>Tareas base de datos:</t>
   </si>
@@ -553,9 +553,6 @@
   </si>
   <si>
     <t>Alberto García                                               1.5h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alberto García                                               </t>
   </si>
 </sst>
 </file>
@@ -803,7 +800,7 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -883,7 +880,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="2" borderId="1" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Énfasis5" xfId="2" builtinId="45"/>
@@ -2620,7 +2616,7 @@
         <v>107</v>
       </c>
       <c r="H48" s="18" t="s">
-        <v>11</v>
+        <v>107</v>
       </c>
       <c r="I48" s="2"/>
     </row>
@@ -2636,7 +2632,7 @@
         <v>106</v>
       </c>
       <c r="H49" s="18" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="I49" s="2"/>
     </row>
@@ -2652,7 +2648,7 @@
         <v>108</v>
       </c>
       <c r="H50" s="18" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="I50" s="2"/>
     </row>
@@ -2668,7 +2664,7 @@
         <v>109</v>
       </c>
       <c r="H51" s="18" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="I51" s="2"/>
     </row>
@@ -2685,7 +2681,7 @@
         <v>110</v>
       </c>
       <c r="H52" s="18" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="I52" s="31"/>
     </row>
@@ -2697,12 +2693,12 @@
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
-      <c r="F53" s="35"/>
+      <c r="F53" s="2"/>
       <c r="G53" s="18" t="s">
         <v>111</v>
       </c>
       <c r="H53" s="18" t="s">
-        <v>21</v>
+        <v>111</v>
       </c>
       <c r="I53" s="2"/>
     </row>
@@ -2718,7 +2714,7 @@
         <v>112</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="I54" s="2"/>
     </row>
@@ -2734,7 +2730,7 @@
         <v>113</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="I55" s="2"/>
     </row>
@@ -2750,7 +2746,7 @@
         <v>114</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="I56" s="2"/>
     </row>
@@ -2766,7 +2762,7 @@
         <v>115</v>
       </c>
       <c r="H57" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I57" s="2"/>
     </row>
@@ -2822,7 +2818,7 @@
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
       <c r="H60" s="18" t="s">
-        <v>11</v>
+        <v>107</v>
       </c>
       <c r="I60" s="18" t="s">
         <v>11</v>
@@ -2838,7 +2834,7 @@
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
       <c r="H61" s="18" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="I61" s="18" t="s">
         <v>13</v>
@@ -2854,7 +2850,7 @@
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
       <c r="H62" s="18" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="I62" s="18" t="s">
         <v>15</v>
@@ -2870,7 +2866,7 @@
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
       <c r="H63" s="18" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="I63" s="18" t="s">
         <v>17</v>
@@ -2886,7 +2882,7 @@
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
       <c r="H64" s="18" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="I64" s="18" t="s">
         <v>19</v>
@@ -2902,7 +2898,7 @@
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
       <c r="H65" s="18" t="s">
-        <v>21</v>
+        <v>111</v>
       </c>
       <c r="I65" s="18" t="s">
         <v>21</v>
@@ -2918,7 +2914,7 @@
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
       <c r="H66" s="18" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="I66" s="18" t="s">
         <v>23</v>
@@ -2934,7 +2930,7 @@
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
       <c r="H67" s="18" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="I67" s="18" t="s">
         <v>25</v>
@@ -2950,7 +2946,7 @@
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
       <c r="H68" s="18" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="I68" s="18" t="s">
         <v>27</v>
@@ -2966,7 +2962,7 @@
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
       <c r="H69" s="18" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="I69" s="18" t="s">
         <v>29</v>
@@ -2994,9 +2990,7 @@
       <c r="E71" s="2"/>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
-      <c r="H71" s="18" t="s">
-        <v>11</v>
-      </c>
+      <c r="H71" s="2"/>
       <c r="I71" s="18" t="s">
         <v>11</v>
       </c>
@@ -3010,9 +3004,7 @@
       <c r="E72" s="2"/>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
-      <c r="H72" s="18" t="s">
-        <v>13</v>
-      </c>
+      <c r="H72" s="2"/>
       <c r="I72" s="18" t="s">
         <v>13</v>
       </c>
@@ -3026,9 +3018,7 @@
       <c r="E73" s="2"/>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
-      <c r="H73" s="18" t="s">
-        <v>15</v>
-      </c>
+      <c r="H73" s="2"/>
       <c r="I73" s="18" t="s">
         <v>15</v>
       </c>
@@ -3042,9 +3032,7 @@
       <c r="E74" s="2"/>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
-      <c r="H74" s="18" t="s">
-        <v>17</v>
-      </c>
+      <c r="H74" s="2"/>
       <c r="I74" s="18" t="s">
         <v>17</v>
       </c>
@@ -3058,9 +3046,7 @@
       <c r="E75" s="31"/>
       <c r="F75" s="31"/>
       <c r="G75" s="31"/>
-      <c r="H75" s="18" t="s">
-        <v>19</v>
-      </c>
+      <c r="H75" s="2"/>
       <c r="I75" s="18" t="s">
         <v>19</v>
       </c>
@@ -3074,9 +3060,7 @@
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
-      <c r="H76" s="18" t="s">
-        <v>21</v>
-      </c>
+      <c r="H76" s="2"/>
       <c r="I76" s="18" t="s">
         <v>21</v>
       </c>
@@ -3090,9 +3074,7 @@
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
-      <c r="H77" s="18" t="s">
-        <v>23</v>
-      </c>
+      <c r="H77" s="2"/>
       <c r="I77" s="18" t="s">
         <v>23</v>
       </c>
@@ -3107,9 +3089,7 @@
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
-      <c r="H78" s="18" t="s">
-        <v>25</v>
-      </c>
+      <c r="H78" s="2"/>
       <c r="I78" s="18" t="s">
         <v>25</v>
       </c>
@@ -3124,9 +3104,7 @@
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
-      <c r="H79" s="18" t="s">
-        <v>27</v>
-      </c>
+      <c r="H79" s="2"/>
       <c r="I79" s="18" t="s">
         <v>27</v>
       </c>
@@ -3141,9 +3119,7 @@
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
-      <c r="H80" s="18" t="s">
-        <v>29</v>
-      </c>
+      <c r="H80" s="2"/>
       <c r="I80" s="18" t="s">
         <v>29</v>
       </c>

</xml_diff>

<commit_message>
Subimos el html y css
</commit_message>
<xml_diff>
--- a/CronogramaHito1_Grupo6.xlsx
+++ b/CronogramaHito1_Grupo6.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Universidad\Proyecto_Computacion_2\proyecto_computacion_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7811A163-75E0-4373-9141-DE1C985F1AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{04A64D97-B4B0-4D5F-BD2D-47C46C51F8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7F42FA1D-32E5-43B4-9CD2-D0CD4F373669}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="106">
   <si>
     <t>Tareas base de datos:</t>
   </si>
@@ -71,61 +71,31 @@
     <t>Requisitos de la base de datos: Identificar y recopilar los requisitos funcionales y no funcionales de la base de datos, incluyendo las entidades, relaciones y atributos clave.</t>
   </si>
   <si>
-    <t>Victor Vega / Alberto García</t>
-  </si>
-  <si>
     <t>Análisis de datos: Realizar un análisis exhaustivo de los datos que se almacenarán en la base de datos para comprender completamente la estructura y las relaciones entre ellos.</t>
   </si>
   <si>
-    <t>Victor Vega</t>
-  </si>
-  <si>
     <t>Modelado conceptual: Utilizar técnicas de modelado conceptual para crear un diagrama de entidad-relación (ER) que represente las entidades, atributos y relaciones de alto nivel en la base de datos.</t>
   </si>
   <si>
-    <t>Samuel Sánchez / Victor Vega</t>
-  </si>
-  <si>
     <t>Normalización de datos: Aplicar las reglas de normalización para eliminar la redundancia y mejorar la integridad de los datos, dividiendo las tablas en formas normales.</t>
   </si>
   <si>
-    <t>Samuel Sánchez</t>
-  </si>
-  <si>
     <t>Diseño lógico: Traducir el modelo conceptual en un modelo lógico, definiendo las tablas, columnas, claves primarias y foráneas, y cualquier otra restricción necesaria.</t>
   </si>
   <si>
-    <t>Samuel Sánchez / Ivan García</t>
-  </si>
-  <si>
     <t>Optimización de consultas: Identificar consultas comunes que se ejecutarán en la base de datos y optimizar el diseño de la base de datos para mejorar el rendimiento de estas consultas.</t>
   </si>
   <si>
-    <t>Ivan García</t>
-  </si>
-  <si>
     <t>Selección de la plataforma de base de datos: Evaluar las necesidades del proyecto y seleccionar la plataforma de base de datos más adecuada, como MySQL, MariaDB u Oracle, basándose en factores como el rendimiento, la escalabilidad y la compatibilidad con el sistema existente.</t>
   </si>
   <si>
-    <t>Ivan García / Jiale Chen</t>
-  </si>
-  <si>
     <t>Implementación física: Crear la base de datos física utilizando el sistema de gestión de bases de datos seleccionado, creando tablas, índices y otras estructuras según el diseño lógico definido.</t>
   </si>
   <si>
-    <t>Jiale Chen</t>
-  </si>
-  <si>
     <t>Pruebas de integración y rendimiento: Realizar pruebas exhaustivas para garantizar que la base de datos funcione según lo previsto, incluyendo pruebas de integración con otras aplicaciones y pruebas de rendimiento para evaluar la velocidad y la escalabilidad.</t>
   </si>
   <si>
-    <t>Jiale Chen / Alberto García</t>
-  </si>
-  <si>
     <t>Documentación y mantenimiento: Documentar el diseño de la base de datos, incluyendo el modelo ER, el modelo lógico, el esquema físico y cualquier otra información relevante, y establecer procesos para el mantenimiento continuo de la base de datos, como la copia de seguridad y la optimización periódica.</t>
-  </si>
-  <si>
-    <t>Alberto García</t>
   </si>
   <si>
     <t>Carga de datos en tablas dinámicamente desde el código.</t>
@@ -1912,7 +1882,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D3" s="27"/>
       <c r="E3" s="27"/>
@@ -1923,10 +1893,10 @@
     </row>
     <row r="4" spans="1:9" s="18" customFormat="1" ht="28.95" customHeight="1">
       <c r="A4" s="28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="D4" s="27"/>
       <c r="E4" s="27"/>
@@ -1937,10 +1907,10 @@
     </row>
     <row r="5" spans="1:9" s="18" customFormat="1" ht="28.95" customHeight="1">
       <c r="A5" s="28" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D5" s="27"/>
       <c r="E5" s="27"/>
@@ -1951,10 +1921,10 @@
     </row>
     <row r="6" spans="1:9" s="18" customFormat="1" ht="28.2" customHeight="1">
       <c r="A6" s="28" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D6" s="27"/>
       <c r="E6" s="27"/>
@@ -1965,10 +1935,10 @@
     </row>
     <row r="7" spans="1:9" s="18" customFormat="1" ht="30.6" customHeight="1">
       <c r="A7" s="28" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D7" s="27"/>
       <c r="E7" s="27"/>
@@ -1979,10 +1949,10 @@
     </row>
     <row r="8" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A8" s="28" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="D8" s="27"/>
       <c r="E8" s="27"/>
@@ -1993,10 +1963,10 @@
     </row>
     <row r="9" spans="1:9" s="18" customFormat="1" ht="28.2" customHeight="1">
       <c r="A9" s="28" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27"/>
@@ -2007,10 +1977,10 @@
     </row>
     <row r="10" spans="1:9" s="18" customFormat="1" ht="28.95" customHeight="1">
       <c r="A10" s="28" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D10" s="27"/>
       <c r="E10" s="27"/>
@@ -2021,10 +1991,10 @@
     </row>
     <row r="11" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A11" s="28" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D11" s="27"/>
       <c r="E11" s="27"/>
@@ -2035,10 +2005,10 @@
     </row>
     <row r="12" spans="1:9" s="18" customFormat="1" ht="29.25" customHeight="1">
       <c r="A12" s="28" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
@@ -2049,7 +2019,7 @@
     </row>
     <row r="13" spans="1:9" s="18" customFormat="1" ht="29.25" customHeight="1">
       <c r="A13" s="33" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C13" s="27"/>
       <c r="D13" s="27"/>
@@ -2061,14 +2031,14 @@
     </row>
     <row r="14" spans="1:9" s="18" customFormat="1" ht="29.25" customHeight="1">
       <c r="A14" s="29" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C14" s="27"/>
       <c r="D14" s="18" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="27"/>
@@ -2077,14 +2047,14 @@
     </row>
     <row r="15" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A15" s="29" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C15" s="27"/>
       <c r="D15" s="18" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="27"/>
@@ -2093,14 +2063,14 @@
     </row>
     <row r="16" spans="1:9" s="18" customFormat="1" ht="28.5" customHeight="1">
       <c r="A16" s="29" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C16" s="27"/>
       <c r="D16" s="18" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="27"/>
@@ -2109,14 +2079,14 @@
     </row>
     <row r="17" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A17" s="29" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C17" s="27"/>
       <c r="D17" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="E17" s="18" t="s">
         <v>99</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>109</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="27"/>
@@ -2125,14 +2095,14 @@
     </row>
     <row r="18" spans="1:9" s="18" customFormat="1" ht="28.5" customHeight="1">
       <c r="A18" s="29" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C18" s="27"/>
       <c r="D18" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="18" t="s">
         <v>100</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>110</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="27"/>
@@ -2141,14 +2111,14 @@
     </row>
     <row r="19" spans="1:9" s="18" customFormat="1" ht="28.5" customHeight="1">
       <c r="A19" s="29" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C19" s="27"/>
       <c r="D19" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="E19" s="18" t="s">
         <v>101</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>111</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="27"/>
@@ -2157,14 +2127,14 @@
     </row>
     <row r="20" spans="1:9" s="18" customFormat="1" ht="29.25" customHeight="1">
       <c r="A20" s="29" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C20" s="27"/>
       <c r="D20" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="E20" s="18" t="s">
         <v>102</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>112</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="27"/>
@@ -2173,14 +2143,14 @@
     </row>
     <row r="21" spans="1:9" s="18" customFormat="1" ht="31.5" customHeight="1">
       <c r="A21" s="29" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C21" s="27"/>
       <c r="D21" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21" s="18" t="s">
         <v>103</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>113</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="27"/>
@@ -2189,14 +2159,14 @@
     </row>
     <row r="22" spans="1:9" s="18" customFormat="1" ht="29.25" customHeight="1">
       <c r="A22" s="29" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C22" s="27"/>
       <c r="D22" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="E22" s="18" t="s">
         <v>104</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>114</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="27"/>
@@ -2205,14 +2175,14 @@
     </row>
     <row r="23" spans="1:9" s="18" customFormat="1" ht="29.25" customHeight="1">
       <c r="A23" s="29" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C23" s="27"/>
       <c r="D23" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="E23" s="18" t="s">
         <v>105</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>115</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="34"/>
@@ -2221,7 +2191,7 @@
     </row>
     <row r="24" spans="1:9" s="18" customFormat="1" ht="29.4" customHeight="1">
       <c r="A24" s="10" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C24" s="27"/>
       <c r="D24" s="27"/>
@@ -2233,15 +2203,15 @@
     </row>
     <row r="25" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A25" s="30" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C25" s="27"/>
       <c r="D25" s="27"/>
       <c r="E25" s="18" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="G25" s="27"/>
       <c r="H25" s="27"/>
@@ -2249,15 +2219,15 @@
     </row>
     <row r="26" spans="1:9" s="18" customFormat="1" ht="30.6" customHeight="1">
       <c r="A26" s="30" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C26" s="27"/>
       <c r="D26" s="27"/>
       <c r="E26" s="18" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="G26" s="27"/>
       <c r="H26" s="27"/>
@@ -2265,15 +2235,15 @@
     </row>
     <row r="27" spans="1:9" s="18" customFormat="1" ht="28.95" customHeight="1">
       <c r="A27" s="30" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C27" s="27"/>
       <c r="D27" s="27"/>
       <c r="E27" s="18" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="G27" s="27"/>
       <c r="H27" s="27"/>
@@ -2281,15 +2251,15 @@
     </row>
     <row r="28" spans="1:9" s="18" customFormat="1" ht="30.6" customHeight="1">
       <c r="A28" s="30" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C28" s="27"/>
       <c r="D28" s="27"/>
       <c r="E28" s="18" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="G28" s="27"/>
       <c r="H28" s="27"/>
@@ -2297,15 +2267,15 @@
     </row>
     <row r="29" spans="1:9" s="18" customFormat="1" ht="30.6" customHeight="1">
       <c r="A29" s="30" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C29" s="27"/>
       <c r="D29" s="27"/>
       <c r="E29" s="18" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="F29" s="18" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="G29" s="27"/>
       <c r="H29" s="27"/>
@@ -2313,15 +2283,15 @@
     </row>
     <row r="30" spans="1:9" s="18" customFormat="1" ht="30.6" customHeight="1">
       <c r="A30" s="30" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C30" s="27"/>
       <c r="D30" s="27"/>
       <c r="E30" s="18" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="G30" s="27"/>
       <c r="H30" s="27"/>
@@ -2329,15 +2299,15 @@
     </row>
     <row r="31" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A31" s="30" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C31" s="27"/>
       <c r="D31" s="27"/>
       <c r="E31" s="18" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="G31" s="27"/>
       <c r="H31" s="27"/>
@@ -2345,15 +2315,15 @@
     </row>
     <row r="32" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A32" s="30" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C32" s="27"/>
       <c r="D32" s="27"/>
       <c r="E32" s="18" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G32" s="27"/>
       <c r="H32" s="27"/>
@@ -2361,15 +2331,15 @@
     </row>
     <row r="33" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A33" s="30" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C33" s="27"/>
       <c r="D33" s="27"/>
       <c r="E33" s="18" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="F33" s="18" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="G33" s="27"/>
       <c r="H33" s="27"/>
@@ -2377,15 +2347,15 @@
     </row>
     <row r="34" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A34" s="30" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C34" s="27"/>
       <c r="D34" s="27"/>
       <c r="E34" s="18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="G34" s="27"/>
       <c r="H34" s="27"/>
@@ -2393,7 +2363,7 @@
     </row>
     <row r="35" spans="1:9" s="21" customFormat="1" ht="157.5" customHeight="1">
       <c r="A35" s="22" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B35" s="23" t="s">
         <v>1</v>
@@ -2422,7 +2392,7 @@
     </row>
     <row r="36" spans="1:9" ht="40.5" customHeight="1">
       <c r="A36" s="6" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -2434,167 +2404,167 @@
     </row>
     <row r="37" spans="1:9" ht="30" customHeight="1">
       <c r="A37" s="8" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="18" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="G37" s="18" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
     </row>
     <row r="38" spans="1:9" ht="30" customHeight="1">
       <c r="A38" s="8" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="18" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="G38" s="18" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
     </row>
     <row r="39" spans="1:9" ht="30" customHeight="1">
       <c r="A39" s="8" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="18" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="G39" s="18" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
     </row>
     <row r="40" spans="1:9" ht="30" customHeight="1">
       <c r="A40" s="8" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
       <c r="F40" s="18" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="G40" s="18" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
     </row>
     <row r="41" spans="1:9" ht="30" customHeight="1">
       <c r="A41" s="8" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
       <c r="F41" s="18" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="G41" s="18" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
     </row>
     <row r="42" spans="1:9" ht="30" customHeight="1">
       <c r="A42" s="8" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="18" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="G42" s="18" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
     </row>
     <row r="43" spans="1:9" ht="30" customHeight="1">
       <c r="A43" s="8" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
       <c r="F43" s="18" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="G43" s="18" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
     </row>
     <row r="44" spans="1:9" ht="30" customHeight="1">
       <c r="A44" s="8" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="18" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G44" s="18" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
     </row>
     <row r="45" spans="1:9" ht="30" customHeight="1">
       <c r="A45" s="8" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
       <c r="F45" s="18" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="G45" s="18" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
     </row>
     <row r="46" spans="1:9" ht="30" customHeight="1">
       <c r="A46" s="12" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
       <c r="F46" s="18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="G46" s="18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
     </row>
     <row r="47" spans="1:9" ht="30" customHeight="1">
       <c r="A47" s="32" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -2606,71 +2576,71 @@
     </row>
     <row r="48" spans="1:9" s="13" customFormat="1" ht="30" customHeight="1">
       <c r="A48" s="8" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
       <c r="G48" s="18" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="H48" s="18" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="I48" s="2"/>
     </row>
     <row r="49" spans="1:9" s="13" customFormat="1" ht="30" customHeight="1">
       <c r="A49" s="9" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
       <c r="G49" s="18" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="H49" s="18" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="I49" s="2"/>
     </row>
     <row r="50" spans="1:9" s="13" customFormat="1" ht="30" customHeight="1">
       <c r="A50" s="8" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
       <c r="G50" s="18" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="H50" s="18" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I50" s="2"/>
     </row>
     <row r="51" spans="1:9" s="13" customFormat="1" ht="30" customHeight="1">
       <c r="A51" s="8" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
       <c r="G51" s="18" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="H51" s="18" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="I51" s="2"/>
     </row>
     <row r="52" spans="1:9" s="11" customFormat="1" ht="30.6" customHeight="1">
       <c r="A52" s="8" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B52" s="13"/>
       <c r="C52" s="31"/>
@@ -2678,16 +2648,16 @@
       <c r="E52" s="31"/>
       <c r="F52" s="2"/>
       <c r="G52" s="18" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="H52" s="18" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="I52" s="31"/>
     </row>
     <row r="53" spans="1:9" s="13" customFormat="1" ht="30.6" customHeight="1">
       <c r="A53" s="8" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B53" s="11"/>
       <c r="C53" s="2"/>
@@ -2695,80 +2665,80 @@
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
       <c r="G53" s="18" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H53" s="18" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="I53" s="2"/>
     </row>
     <row r="54" spans="1:9" s="13" customFormat="1" ht="30" customHeight="1">
       <c r="A54" s="8" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
       <c r="G54" s="18" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="I54" s="2"/>
     </row>
     <row r="55" spans="1:9" s="13" customFormat="1" ht="30.6" customHeight="1">
       <c r="A55" s="8" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
       <c r="G55" s="18" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="I55" s="2"/>
     </row>
     <row r="56" spans="1:9" s="13" customFormat="1" ht="30" customHeight="1">
       <c r="A56" s="14" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
       <c r="G56" s="18" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="I56" s="2"/>
     </row>
     <row r="57" spans="1:9" s="13" customFormat="1" ht="30.6" customHeight="1">
       <c r="A57" s="14" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
       <c r="G57" s="18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="H57" s="18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="I57" s="2"/>
     </row>
     <row r="58" spans="1:9" s="21" customFormat="1" ht="198.75" customHeight="1">
       <c r="A58" s="25" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="B58" s="21" t="s">
         <v>1</v>
@@ -2797,7 +2767,7 @@
     </row>
     <row r="59" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1">
       <c r="A59" s="17" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
@@ -2809,7 +2779,7 @@
     </row>
     <row r="60" spans="1:9" s="13" customFormat="1" ht="30" customHeight="1">
       <c r="A60" s="15" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B60"/>
       <c r="C60" s="2"/>
@@ -2818,15 +2788,15 @@
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
       <c r="H60" s="18" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="I60" s="18" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61" spans="1:9" s="13" customFormat="1" ht="30.6" customHeight="1">
       <c r="A61" s="15" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
@@ -2834,15 +2804,15 @@
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
       <c r="H61" s="18" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="I61" s="18" t="s">
-        <v>13</v>
+        <v>96</v>
       </c>
     </row>
     <row r="62" spans="1:9" s="13" customFormat="1" ht="30.6" customHeight="1">
       <c r="A62" s="15" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
@@ -2850,15 +2820,15 @@
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
       <c r="H62" s="18" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I62" s="18" t="s">
-        <v>15</v>
+        <v>98</v>
       </c>
     </row>
     <row r="63" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A63" s="15" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
@@ -2866,15 +2836,15 @@
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
       <c r="H63" s="18" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="I63" s="18" t="s">
-        <v>17</v>
+        <v>99</v>
       </c>
     </row>
     <row r="64" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A64" s="15" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
@@ -2882,15 +2852,15 @@
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
       <c r="H64" s="18" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="I64" s="18" t="s">
-        <v>19</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A65" s="15" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -2898,15 +2868,15 @@
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
       <c r="H65" s="18" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="I65" s="18" t="s">
-        <v>21</v>
+        <v>101</v>
       </c>
     </row>
     <row r="66" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A66" s="15" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
@@ -2914,15 +2884,15 @@
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
       <c r="H66" s="18" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="I66" s="18" t="s">
-        <v>23</v>
+        <v>102</v>
       </c>
     </row>
     <row r="67" spans="1:9" s="16" customFormat="1" ht="30" customHeight="1">
       <c r="A67" s="15" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
@@ -2930,15 +2900,15 @@
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
       <c r="H67" s="18" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="I67" s="18" t="s">
-        <v>25</v>
+        <v>103</v>
       </c>
     </row>
     <row r="68" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A68" s="15" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
@@ -2946,15 +2916,15 @@
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
       <c r="H68" s="18" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="I68" s="18" t="s">
-        <v>27</v>
+        <v>104</v>
       </c>
     </row>
     <row r="69" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A69" s="15" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
@@ -2962,15 +2932,15 @@
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
       <c r="H69" s="18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="I69" s="18" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
     </row>
     <row r="70" spans="1:9" s="18" customFormat="1" ht="30.6" customHeight="1">
       <c r="A70" s="32" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
@@ -2982,7 +2952,7 @@
     </row>
     <row r="71" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A71" s="15" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B71" s="3"/>
       <c r="C71" s="2"/>
@@ -2992,12 +2962,12 @@
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="18" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
     </row>
     <row r="72" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A72" s="15" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
@@ -3006,12 +2976,12 @@
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="18" t="s">
-        <v>13</v>
+        <v>96</v>
       </c>
     </row>
     <row r="73" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A73" s="15" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
@@ -3020,12 +2990,12 @@
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="18" t="s">
-        <v>15</v>
+        <v>98</v>
       </c>
     </row>
     <row r="74" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A74" s="15" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
@@ -3034,12 +3004,12 @@
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="18" t="s">
-        <v>17</v>
+        <v>99</v>
       </c>
     </row>
     <row r="75" spans="1:9" s="16" customFormat="1" ht="30" customHeight="1">
       <c r="A75" s="15" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C75" s="31"/>
       <c r="D75" s="31"/>
@@ -3048,12 +3018,12 @@
       <c r="G75" s="31"/>
       <c r="H75" s="2"/>
       <c r="I75" s="18" t="s">
-        <v>19</v>
+        <v>100</v>
       </c>
     </row>
     <row r="76" spans="1:9" s="16" customFormat="1" ht="30" customHeight="1">
       <c r="A76" s="15" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
@@ -3062,12 +3032,12 @@
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="18" t="s">
-        <v>21</v>
+        <v>101</v>
       </c>
     </row>
     <row r="77" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A77" s="15" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
@@ -3076,12 +3046,12 @@
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="18" t="s">
-        <v>23</v>
+        <v>102</v>
       </c>
     </row>
     <row r="78" spans="1:9" s="16" customFormat="1" ht="30" customHeight="1">
       <c r="A78" s="15" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B78" s="15"/>
       <c r="C78" s="2"/>
@@ -3091,12 +3061,12 @@
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="18" t="s">
-        <v>25</v>
+        <v>103</v>
       </c>
     </row>
     <row r="79" spans="1:9" s="16" customFormat="1" ht="30.6" customHeight="1">
       <c r="A79" s="15" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B79" s="15"/>
       <c r="C79" s="2"/>
@@ -3106,12 +3076,12 @@
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="18" t="s">
-        <v>27</v>
+        <v>104</v>
       </c>
     </row>
     <row r="80" spans="1:9" s="16" customFormat="1" ht="30" customHeight="1">
       <c r="A80" s="15" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B80" s="15"/>
       <c r="C80" s="2"/>
@@ -3121,7 +3091,7 @@
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="18" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="18">

</xml_diff>